<commit_message>
Planogram update 2026-05-12 00:30
</commit_message>
<xml_diff>
--- a/docs/planogram.xlsx
+++ b/docs/planogram.xlsx
@@ -12860,7 +12860,7 @@
     <t>קרט/יום</t>
   </si>
   <si>
-    <t>ימים נותרים</t>
+    <t>יספיק ל (ימים)</t>
   </si>
   <si>
     <t>‬יוגורט יווני200 ג(6)'‭</t>
@@ -19702,7 +19702,7 @@
     <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:5" s="91" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Planogram update 2026-05-12 16:48
</commit_message>
<xml_diff>
--- a/docs/planogram.xlsx
+++ b/docs/planogram.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1318" uniqueCount="685">
   <si>
     <t>דגים  ·  הזמנות/d: 1481 | מכר: 10.8 PAL/d  ·  פעיל: 40 | אפס מלאי: 15   ║   כל המחסנים: 4586 הזמנות/d</t>
   </si>
@@ -36,7 +36,7 @@
     <t>SANTA BREMOR Fish</t>
   </si>
   <si>
-    <t>BI עודכן: 12.05, 09:47</t>
+    <t>BI עודכן: 12.05, 16:44</t>
   </si>
   <si>
     <t>12 BAYS</t>
@@ -133,7 +133,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 36.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 36.4 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -257,7 +257,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 172.1 קרט | 0.6 PAL
+      <t xml:space="preserve">AVG/d: 172.1 | 0.6 PAL
 </t>
     </r>
     <r>
@@ -381,7 +381,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 55.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 55.4 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -505,7 +505,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 42.8 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 42.8 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -632,7 +632,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 13.0 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 13.0 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -756,7 +756,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 80.5 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 80.5 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -889,7 +889,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 36.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 36.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -1022,7 +1022,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 42.8 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 42.8 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -1164,7 +1164,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 51.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 51.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -1297,7 +1297,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 28.6 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 28.6 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -1430,7 +1430,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 119.4 קרט | 0.5 PAL
+      <t xml:space="preserve">AVG/d: 119.4 | 0.5 PAL
 </t>
     </r>
     <r>
@@ -1570,7 +1570,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 59.6 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 59.6 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -1694,7 +1694,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 49.3 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 49.3 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -1852,7 +1852,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 40.4 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 40.4 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -1979,7 +1979,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 15.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -2119,7 +2119,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 59.2 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 59.2 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -2255,7 +2255,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 23.7 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 23.7 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -2364,7 +2364,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 24.6 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 24.6 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -2506,7 +2506,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 33.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 33.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -2630,7 +2630,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 66.3 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 66.3 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -2779,7 +2779,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 37.1 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 37.1 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -2903,7 +2903,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 68.9 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 68.9 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -3036,7 +3036,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 32.3 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 32.3 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -3167,7 +3167,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 74.2 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 74.2 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -3295,7 +3295,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 60.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 60.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -3417,7 +3417,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 13.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 13.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -3550,7 +3550,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 56.5 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 56.5 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -3668,7 +3668,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 25.6 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 25.6 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -3786,7 +3786,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 20.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 20.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -3919,7 +3919,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 38.7 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 38.7 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -4052,7 +4052,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 110.5 קרט | 0.5 PAL
+      <t xml:space="preserve">AVG/d: 110.5 | 0.5 PAL
 </t>
     </r>
     <r>
@@ -4185,7 +4185,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 101.1 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 101.1 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -4303,7 +4303,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 28.3 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 28.3 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -4436,7 +4436,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 72.1 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 72.1 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -4578,7 +4578,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 69.1 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 69.1 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -4705,7 +4705,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 8.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 8.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -4836,7 +4836,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 70.7 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 70.7 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -4987,7 +4987,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 43.5 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 43.5 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -5129,7 +5129,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 25.3 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 25.3 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -5271,7 +5271,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 73.1 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 73.1 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -5404,7 +5404,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 2.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 2.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -5537,7 +5537,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 25.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 25.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -5670,7 +5670,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 3.2 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 3.2 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -5801,7 +5801,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 38.6 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 38.6 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -6076,7 +6076,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 25.1 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 25.1 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -6218,7 +6218,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 5.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 5.4 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -6351,7 +6351,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 18.1 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 18.1 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -6484,7 +6484,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 60.8 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 60.8 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -6617,7 +6617,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 93.7 קרט | 0.5 PAL
+      <t xml:space="preserve">AVG/d: 93.7 | 0.5 PAL
 </t>
     </r>
     <r>
@@ -6757,7 +6757,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 96.6 קרט | 0.7 PAL
+      <t xml:space="preserve">AVG/d: 96.6 | 0.7 PAL
 </t>
     </r>
     <r>
@@ -6821,7 +6821,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">פק"ע 31/05/26 (19d) 2קרט
+      <t xml:space="preserve">פק"ע 31/05/26 (19d) 17קרט
 </t>
     </r>
   </si>
@@ -6866,7 +6866,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.8 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 15.8 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -6999,7 +6999,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 64.5 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 64.5 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -7141,7 +7141,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 37.5 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 37.5 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -7277,7 +7277,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 14.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 14.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -7419,7 +7419,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 36.1 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 36.1 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -7546,7 +7546,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 8.2 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 8.2 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -7686,7 +7686,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 114.0 קרט | 0.9 PAL
+      <t xml:space="preserve">AVG/d: 114.0 | 0.9 PAL
 </t>
     </r>
     <r>
@@ -7826,7 +7826,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 92.7 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 92.7 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -7959,7 +7959,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 128.1 קרט | 0.8 PAL
+      <t xml:space="preserve">AVG/d: 128.1 | 0.8 PAL
 </t>
     </r>
     <r>
@@ -8092,7 +8092,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 75.8 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 75.8 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -8216,7 +8216,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 55.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 55.4 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -8322,7 +8322,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 65.8 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 65.8 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -8446,7 +8446,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 135.8 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 135.8 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -8553,7 +8553,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 100.8 קרט
+      <t xml:space="preserve">AVG/d: 100.8
 </t>
     </r>
     <r>
@@ -8677,7 +8677,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 6.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 6.0 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -8819,7 +8819,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 7.2 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 7.2 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -8952,7 +8952,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 7.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 7.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -9070,7 +9070,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 8.2 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 8.2 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -9212,7 +9212,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 33.8 קרט | 0.5 PAL
+      <t xml:space="preserve">AVG/d: 33.8 | 0.5 PAL
 </t>
     </r>
     <r>
@@ -9468,7 +9468,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 68.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 68.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -9592,7 +9592,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 85.0 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 85.0 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -9716,7 +9716,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 82.0 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 82.0 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -9840,7 +9840,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 50.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 50.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -9964,7 +9964,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 46.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 46.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -10088,7 +10088,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 57.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 57.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -10212,7 +10212,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 63.0 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 63.0 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -10336,7 +10336,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 64.0 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 64.0 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -10470,7 +10470,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 77.0 קרט | 0.5 PAL
+      <t xml:space="preserve">AVG/d: 77.0 | 0.5 PAL
 </t>
     </r>
     <r>
@@ -10594,7 +10594,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 59.0 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 59.0 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -10718,7 +10718,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 69.0 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 69.0 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -10842,7 +10842,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 66.0 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 66.0 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -10966,7 +10966,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 90.0 קרט | 0.5 PAL
+      <t xml:space="preserve">AVG/d: 90.0 | 0.5 PAL
 </t>
     </r>
     <r>
@@ -11090,7 +11090,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 38.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 38.0 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -11223,7 +11223,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 38.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 38.0 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -11332,7 +11332,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 32.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 32.0 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -11456,7 +11456,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 58.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 58.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -11520,7 +11520,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">פק"ע 26/08/26 (106d) 77קרט
+      <t xml:space="preserve">פק"ע 26/08/26 (106d) 127קרט
 </t>
     </r>
     <r>
@@ -11589,7 +11589,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 60.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 60.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -11731,7 +11731,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 44.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 44.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -11873,7 +11873,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 77.0 קרט | 0.4 PAL
+      <t xml:space="preserve">AVG/d: 77.0 | 0.4 PAL
 </t>
     </r>
     <r>
@@ -12077,7 +12077,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 222.9 קרט | 1.0 PAL
+      <t xml:space="preserve">AVG/d: 222.9 | 1.0 PAL
 </t>
     </r>
     <r>
@@ -12208,7 +12208,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 61.4 קרט | 0.3 PAL
+      <t xml:space="preserve">AVG/d: 61.4 | 0.3 PAL
 </t>
     </r>
     <r>
@@ -12332,7 +12332,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 13.2 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 13.2 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -12465,7 +12465,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 6.4 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 6.4 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -12589,7 +12589,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 5.9 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 5.8 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -12635,7 +12635,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">יספיק: 129 ימים
+      <t xml:space="preserve">יספיק: 133 ימים
 </t>
     </r>
     <r>
@@ -12653,7 +12653,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">פק"ע 20/07/26 (69d) 286קרט
+      <t xml:space="preserve">פק"ע 20/07/26 (69d) 287קרט
 </t>
     </r>
     <r>
@@ -12722,7 +12722,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 7.5 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 7.5 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -12846,7 +12846,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 6.8 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 6.8 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -12955,7 +12955,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 34.8 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 34.8 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -13073,7 +13073,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 24.0 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 24.0 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -13191,7 +13191,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 14.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 14.7 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -13237,7 +13237,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">יספיק: 58 ימים
+      <t xml:space="preserve">יספיק: 59 ימים
 </t>
     </r>
     <r>
@@ -13255,7 +13255,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">פק"ע 18/01/27 (251d) 20קרט
+      <t xml:space="preserve">פק"ע 18/01/27 (251d) 22קרט
 </t>
     </r>
     <r>
@@ -13318,7 +13318,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 13.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 13.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -13445,7 +13445,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 14.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 14.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -13554,7 +13554,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 18.1 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 18.1 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -13672,7 +13672,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.1 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 15.1 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -13799,7 +13799,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 14.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 14.2 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -13845,7 +13845,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">יספיק: 44 ימים
+      <t xml:space="preserve">יספיק: 45 ימים
 </t>
     </r>
     <r>
@@ -13863,7 +13863,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">פק"ע 18/01/27 (251d) 41קרט
+      <t xml:space="preserve">פק"ע 18/01/27 (251d) 42קרט
 </t>
     </r>
     <r>
@@ -13926,7 +13926,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.9 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 15.9 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -14044,7 +14044,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 12.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 12.0 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -14177,7 +14177,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 17.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 17.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -14310,7 +14310,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.3 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 15.3 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -14443,7 +14443,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 14.7 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 14.7 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -14576,7 +14576,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 14.6 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -14622,7 +14622,7 @@
         <sz val="9"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">יספיק: 60 ימים
+      <t xml:space="preserve">יספיק: 61 ימים
 </t>
     </r>
     <r>
@@ -14640,7 +14640,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">פק"ע 09/11/26 (181d) 51קרט
+      <t xml:space="preserve">פק"ע 09/11/26 (181d) 52קרט
 </t>
     </r>
     <r>
@@ -14709,7 +14709,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 70.1 קרט | 0.9 PAL
+      <t xml:space="preserve">AVG/d: 70.1 | 0.9 PAL
 </t>
     </r>
     <r>
@@ -14833,7 +14833,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 68.5 קרט | 0.8 PAL
+      <t xml:space="preserve">AVG/d: 68.5 | 0.8 PAL
 </t>
     </r>
     <r>
@@ -14957,7 +14957,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 84.5 קרט | 1.0 PAL
+      <t xml:space="preserve">AVG/d: 84.5 | 1.0 PAL
 </t>
     </r>
     <r>
@@ -15081,7 +15081,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 143.2 קרט | 1.8 PAL
+      <t xml:space="preserve">AVG/d: 143.2 | 1.8 PAL
 </t>
     </r>
     <r>
@@ -15214,7 +15214,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 8.0 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 8.0 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -15338,7 +15338,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 10.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 10.4 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -15447,7 +15447,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 3.5 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 3.5 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -15574,7 +15574,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 12.3 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 12.3 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -15716,7 +15716,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 2.6 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 2.6 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -15867,7 +15867,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 2.9 קרט | 0.0 PAL
+      <t xml:space="preserve">AVG/d: 2.9 | 0.0 PAL
 </t>
     </r>
     <r>
@@ -16009,7 +16009,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 2.4 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 2.4 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -16133,7 +16133,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 6.7 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 6.7 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -16257,7 +16257,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 9.2 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 9.2 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -16390,7 +16390,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 15.3 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 15.3 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -16574,7 +16574,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 5.3 קרט | 0.1 PAL
+      <t xml:space="preserve">AVG/d: 5.3 | 0.1 PAL
 </t>
     </r>
     <r>
@@ -16707,7 +16707,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 16.8 קרט | 0.2 PAL
+      <t xml:space="preserve">AVG/d: 16.8 | 0.2 PAL
 </t>
     </r>
     <r>
@@ -16856,7 +16856,7 @@
         <sz val="8"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">AVG/d: 44.0 קרט | 0.6 PAL
+      <t xml:space="preserve">AVG/d: 44.0 | 0.6 PAL
 </t>
     </r>
     <r>
@@ -17960,28 +17960,229 @@
     <t>מלאי (קרטון)</t>
   </si>
   <si>
+    <t>‬חמאה200 FERMA 82.5% ג(20)'‭</t>
+  </si>
+  <si>
+    <t>029</t>
+  </si>
+  <si>
+    <t>721</t>
+  </si>
+  <si>
+    <t>‬דג וובלה מיובש‭</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>‬חמאה200 ROSHEN 82.5% ג(24)'‭</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
     <t>‬פילה סלמון מעושן פרוס מצונן100 גרםNP(10) ‭</t>
   </si>
   <si>
     <t>036</t>
   </si>
   <si>
+    <t>‬סלט איקרה ורודה 180 גרםNP(6) ‭</t>
+  </si>
+  <si>
+    <t>0301</t>
+  </si>
+  <si>
+    <t>‬בסגנון קוויאר אדום כדורי דג פורל230 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>717</t>
+  </si>
+  <si>
+    <t>‬דג לש 'מיובש‭</t>
+  </si>
+  <si>
+    <t>719</t>
+  </si>
+  <si>
+    <t>‬דג סודאק מיובש‭</t>
+  </si>
+  <si>
+    <t>724</t>
+  </si>
+  <si>
+    <t>‬דג לש 'מעושן‭</t>
+  </si>
+  <si>
+    <t>‬שמנת 30% SMETANA שומן200 ג(12) '‭</t>
+  </si>
+  <si>
+    <t>021</t>
+  </si>
+  <si>
     <t>‬פילה פורל מעושן פרוס מצונן100 גרםNP(10) ‭</t>
   </si>
   <si>
+    <t>‬משקה חלבי0.5 (RIAZENKA) ל(6) '‭</t>
+  </si>
+  <si>
+    <t>‬ GURMANגבינה אנלוגי מעושנת150 ג(14)'‭</t>
+  </si>
+  <si>
+    <t>028</t>
+  </si>
+  <si>
+    <t>‬סלט איקרה לבנה 180 גרםNP(6) ‭</t>
+  </si>
+  <si>
+    <t>‬גבינה מותכת 28%  שומן160 גרם(6) SVALYA ‭</t>
+  </si>
+  <si>
+    <t>020</t>
+  </si>
+  <si>
+    <t>‬שמנת 15% SMETANA שומן350 ג(12)'‭</t>
+  </si>
+  <si>
+    <t>‬טבורוג 350 5% גרם(8) (SVALYA) ‭</t>
+  </si>
+  <si>
+    <t>‬בלינצ'ס במילוי גבינת טבורוג מוקפא360 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>019</t>
+  </si>
+  <si>
+    <t>‬סלט אצות ים-צ'וקה150 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>030</t>
+  </si>
+  <si>
+    <t>‬בלינצ'ס) פרווה (במילוי דובדבן מוקפא360 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬טבורוג 800 5% גרם(4) (SVALYA) ‭</t>
+  </si>
+  <si>
+    <t>‬יוגורט יווני200 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬בצק שמרים עלים מרודד מוקפא450 ג(7)'‭</t>
+  </si>
+  <si>
+    <t>‬בצק עלים מרודד מוקפא450 ג(7)'‭</t>
+  </si>
+  <si>
     <t>‬פילה סלמון מעושן פרוס מצונן250 גרםNP(9) ‭</t>
   </si>
   <si>
+    <t>‬בלינצ'ס) פרווה (במילוי תפו"א ופטריות מוקפא420 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬כיסונים במילוי דובדבנים מוקפאים450 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬ SVALYAגבינה אנלוגי150 ג(18)'‭</t>
+  </si>
+  <si>
+    <t>‬כיסונים" פרווה "במילוי תפו"א ובצל מוקפאים450 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬כיסונים" פרווה "במילוי תפו"א ופטריות מוקפאים450 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬כיסונים במילוי גבינת טבורוג מוקפאים450 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬לביבות גבינת טבורוג מוקפאות450 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬סלט אצות ים מוחמצות200 ג(12)'‭</t>
+  </si>
+  <si>
     <t>‬פילה מקרל מומלח בעישון חם מצונן150 גרם8) NP) ‭</t>
   </si>
   <si>
+    <t>‬קפיר0.9 (KEFIR) ל(10) '‭</t>
+  </si>
+  <si>
+    <t>‬יוגורט יווני עם דובדבן150 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬בצק שמרים מרודד מוקפא450 ג(7)'‭</t>
+  </si>
+  <si>
+    <t>‬בלינצ'ס) פרווה (במילוי תפו"ע וקינמון מוקפא360 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬טבורוג 350 3% גרם(8) (SVALYA) ‭</t>
+  </si>
+  <si>
+    <t>‬ ROSSIYSKIYגבינה אנלוגי150 ג(18)'‭</t>
+  </si>
+  <si>
+    <t>‬דייסת אורז עם משמש200 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬דייסת שיבולת שועל200 ג(6)'‭</t>
+  </si>
+  <si>
+    <t>‬דייסת סולת עם תותי בר200 ג(6)'‭</t>
+  </si>
+  <si>
     <t>‬פילה פורל מעושן פרוס מצונן250 גרםNP(9) ‭</t>
   </si>
   <si>
+    <t>755</t>
+  </si>
+  <si>
+    <t>‬ GURMANגבינה אנלוגי מעושנת4)  LITA) ‭</t>
+  </si>
+  <si>
+    <t>025</t>
+  </si>
+  <si>
+    <t>‬טבורוג250 5% ג(6) (SVALYA)'‭</t>
+  </si>
+  <si>
+    <t>728</t>
+  </si>
+  <si>
+    <t>‬דג ז'אריך מעושן‭</t>
+  </si>
+  <si>
+    <t>727</t>
+  </si>
+  <si>
+    <t>‬דג ז'אריך מיובש‭</t>
+  </si>
+  <si>
+    <t>‬סלט אצות ים מוחמצות ומתובלות עם גזר200 ג(12)'‭</t>
+  </si>
+  <si>
+    <t>‬פילה פורל מעושן מצונן200 גרםNP(5) ‭</t>
+  </si>
+  <si>
     <t>‬פילה סלמון מעושן מצונן200 גרםNP(5) ‭</t>
   </si>
   <si>
-    <t>‬פילה פורל מעושן מצונן200 גרםNP(5) ‭</t>
+    <t>725</t>
+  </si>
+  <si>
+    <t>‬דג צ'חון מעושן‭</t>
+  </si>
+  <si>
+    <t>‬קפיר500 (KEFIR) ג(10)'‭</t>
+  </si>
+  <si>
+    <t>726</t>
+  </si>
+  <si>
+    <t>‬דג צ'חון מיובש‭</t>
+  </si>
+  <si>
+    <t>‬בלינצ'ס) פרווה (במילוי ממרח קקאו-אגוזי לוז מוקפא360 ג(6)‭</t>
   </si>
   <si>
     <t>1113</t>
@@ -17996,6 +18197,12 @@
     <t>‬פילה מקרל מומלח בעישון חם עם פלפל שחור גרוס150 גרם8) NP) ‭</t>
   </si>
   <si>
+    <t>‬ ROSSIYSKIYגבינה אנלוגי5)  LITA) ‭</t>
+  </si>
+  <si>
+    <t>‬ SVALYAגבינה אנלוגי5) LITA) ‭</t>
+  </si>
+  <si>
     <t>1114</t>
   </si>
   <si>
@@ -18014,6 +18221,21 @@
     <t>‬פרוסות דג שיבוט אלבין מיובש ומומלח100 ג(50)'‭</t>
   </si>
   <si>
+    <t>‬טבורוג 350 0.5% גרם(8) (SVALYA) ‭</t>
+  </si>
+  <si>
+    <t>‬ DVAROגבינה אנלוגי150 ג(18)'‭</t>
+  </si>
+  <si>
+    <t>664</t>
+  </si>
+  <si>
+    <t>‬גבינה אנלוגי מעושנת1 SNACKS ק"ג4) LITA) ‭</t>
+  </si>
+  <si>
+    <t>‬סלט אצות ים מוחמצות עם בצל ופפריקה מתוקה200 ג(12)'‭</t>
+  </si>
+  <si>
     <t>1119</t>
   </si>
   <si>
@@ -18050,15 +18272,9 @@
     <t>יספיק ל (ימים)</t>
   </si>
   <si>
-    <t>‬יוגורט יווני עם דובדבן150 ג(6)'‭</t>
-  </si>
-  <si>
     <t>‬עוגת NAPOLEON שכבות בצק עלים וקרם וניל1 ק"ג(4)‭</t>
   </si>
   <si>
-    <t>‬טבורוג 800 5% גרם(4) (SVALYA) ‭</t>
-  </si>
-  <si>
     <t>‬גבינה מותכת  GOUDA שומן150 17% גרם12) PRESIDENT)‭</t>
   </si>
   <si>
@@ -18068,9 +18284,6 @@
     <t>‬גבינה מותכת  CREAMY שומן150 18.3% גרם12) PRESIDENT)‭</t>
   </si>
   <si>
-    <t>‬קפיר0.9 (KEFIR) ל(10) '‭</t>
-  </si>
-  <si>
     <t>‬שמנת חמוצה טבעית 30% שומן300 גרם8) PRESIDENT)‭</t>
   </si>
   <si>
@@ -18078,9 +18291,6 @@
   </si>
   <si>
     <t>‬גבינה קשה למחצה HOLLAND שומן160 24.5%  גרם14) PRESIDENT) ‭</t>
-  </si>
-  <si>
-    <t>‬דייסת שיבולת שועל200 ג(6)'‭</t>
   </si>
   <si>
     <t>‬שמנת חמוצה טבעית 20% שומן300 גרם8) PRESIDENT)‭</t>
@@ -24514,7 +24724,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -24539,7 +24749,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="81" t="s">
-        <v>77</v>
+        <v>264</v>
       </c>
       <c r="B2" s="81" t="s">
         <v>570</v>
@@ -24548,231 +24758,987 @@
         <v>571</v>
       </c>
       <c r="D2" s="82">
-        <v>2884</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="83" t="s">
-        <v>80</v>
+        <v>572</v>
       </c>
       <c r="B3" s="83" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C3" s="83" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D3" s="84">
-        <v>1262</v>
+        <v>4302</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="81" t="s">
-        <v>82</v>
+        <v>228</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C4" s="81" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="D4" s="82">
-        <v>632</v>
+        <v>4140</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="83" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D5" s="84">
-        <v>492</v>
+        <v>2884</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="81" t="s">
-        <v>84</v>
+        <v>567</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="C6" s="81" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D6" s="82">
-        <v>362</v>
+        <v>2326</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="83" t="s">
-        <v>86</v>
+        <v>560</v>
       </c>
       <c r="B7" s="83" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D7" s="84">
-        <v>327</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="81" t="s">
-        <v>88</v>
+        <v>582</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="C8" s="81" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D8" s="82">
-        <v>327</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="83" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B9" s="83" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="C9" s="83" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
       <c r="D9" s="84">
-        <v>250</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="81" t="s">
-        <v>92</v>
+        <v>586</v>
       </c>
       <c r="B10" s="81" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="C10" s="81" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D10" s="82">
-        <v>247</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="83" t="s">
-        <v>582</v>
+        <v>424</v>
       </c>
       <c r="B11" s="83" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="C11" s="83" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="D11" s="84">
-        <v>220</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="81" t="s">
-        <v>584</v>
+        <v>80</v>
       </c>
       <c r="B12" s="81" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="C12" s="81" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D12" s="82">
-        <v>220</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="83" t="s">
-        <v>586</v>
+        <v>422</v>
       </c>
       <c r="B13" s="83" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="C13" s="83" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="D13" s="84">
-        <v>200</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="81" t="s">
-        <v>588</v>
+        <v>454</v>
       </c>
       <c r="B14" s="81" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="C14" s="81" t="s">
-        <v>580</v>
+        <v>593</v>
       </c>
       <c r="D14" s="82">
-        <v>150</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="83" t="s">
-        <v>590</v>
+        <v>565</v>
       </c>
       <c r="B15" s="83" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C15" s="83" t="s">
         <v>580</v>
       </c>
       <c r="D15" s="84">
-        <v>110</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="81" t="s">
-        <v>592</v>
+        <v>464</v>
       </c>
       <c r="B16" s="81" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="C16" s="81" t="s">
-        <v>580</v>
+        <v>596</v>
       </c>
       <c r="D16" s="82">
-        <v>100</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="83" t="s">
-        <v>594</v>
+        <v>419</v>
       </c>
       <c r="B17" s="83" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="C17" s="83" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="D17" s="84">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="81" t="s">
+        <v>461</v>
+      </c>
+      <c r="B18" s="81" t="s">
+        <v>598</v>
+      </c>
+      <c r="C18" s="81" t="s">
+        <v>596</v>
+      </c>
+      <c r="D18" s="82">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="83" t="s">
+        <v>282</v>
+      </c>
+      <c r="B19" s="83" t="s">
+        <v>599</v>
+      </c>
+      <c r="C19" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D19" s="84">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="81" t="s">
+        <v>558</v>
+      </c>
+      <c r="B20" s="81" t="s">
+        <v>601</v>
+      </c>
+      <c r="C20" s="81" t="s">
+        <v>602</v>
+      </c>
+      <c r="D20" s="82">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="83" t="s">
+        <v>285</v>
+      </c>
+      <c r="B21" s="83" t="s">
+        <v>603</v>
+      </c>
+      <c r="C21" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D21" s="84">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="81" t="s">
+        <v>459</v>
+      </c>
+      <c r="B22" s="81" t="s">
+        <v>604</v>
+      </c>
+      <c r="C22" s="81" t="s">
+        <v>596</v>
+      </c>
+      <c r="D22" s="82">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="83" t="s">
+        <v>432</v>
+      </c>
+      <c r="B23" s="83" t="s">
+        <v>605</v>
+      </c>
+      <c r="C23" s="83" t="s">
+        <v>589</v>
+      </c>
+      <c r="D23" s="84">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="81" t="s">
+        <v>311</v>
+      </c>
+      <c r="B24" s="81" t="s">
+        <v>606</v>
+      </c>
+      <c r="C24" s="81" t="s">
+        <v>600</v>
+      </c>
+      <c r="D24" s="82">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="83" t="s">
+        <v>305</v>
+      </c>
+      <c r="B25" s="83" t="s">
+        <v>607</v>
+      </c>
+      <c r="C25" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D25" s="84">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="81" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="81" t="s">
+        <v>608</v>
+      </c>
+      <c r="C26" s="81" t="s">
+        <v>578</v>
+      </c>
+      <c r="D26" s="82">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="83" t="s">
+        <v>287</v>
+      </c>
+      <c r="B27" s="83" t="s">
+        <v>609</v>
+      </c>
+      <c r="C27" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D27" s="84">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="81" t="s">
+        <v>294</v>
+      </c>
+      <c r="B28" s="81" t="s">
+        <v>610</v>
+      </c>
+      <c r="C28" s="81" t="s">
+        <v>600</v>
+      </c>
+      <c r="D28" s="82">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="83" t="s">
+        <v>448</v>
+      </c>
+      <c r="B29" s="83" t="s">
+        <v>611</v>
+      </c>
+      <c r="C29" s="83" t="s">
+        <v>593</v>
+      </c>
+      <c r="D29" s="84">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="81" t="s">
+        <v>297</v>
+      </c>
+      <c r="B30" s="81" t="s">
+        <v>612</v>
+      </c>
+      <c r="C30" s="81" t="s">
+        <v>600</v>
+      </c>
+      <c r="D30" s="82">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="83" t="s">
+        <v>303</v>
+      </c>
+      <c r="B31" s="83" t="s">
+        <v>613</v>
+      </c>
+      <c r="C31" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D31" s="84">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="81" t="s">
+        <v>299</v>
+      </c>
+      <c r="B32" s="81" t="s">
+        <v>614</v>
+      </c>
+      <c r="C32" s="81" t="s">
+        <v>600</v>
+      </c>
+      <c r="D32" s="82">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="83" t="s">
+        <v>301</v>
+      </c>
+      <c r="B33" s="83" t="s">
+        <v>615</v>
+      </c>
+      <c r="C33" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D33" s="84">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="81" t="s">
+        <v>505</v>
+      </c>
+      <c r="B34" s="81" t="s">
+        <v>616</v>
+      </c>
+      <c r="C34" s="81" t="s">
+        <v>602</v>
+      </c>
+      <c r="D34" s="82">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="83" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" s="85" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="85" t="s">
+      <c r="B35" s="83" t="s">
+        <v>617</v>
+      </c>
+      <c r="C35" s="83" t="s">
+        <v>578</v>
+      </c>
+      <c r="D35" s="84">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="81" t="s">
+        <v>416</v>
+      </c>
+      <c r="B36" s="81" t="s">
+        <v>618</v>
+      </c>
+      <c r="C36" s="81" t="s">
+        <v>589</v>
+      </c>
+      <c r="D36" s="82">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="83" t="s">
+        <v>434</v>
+      </c>
+      <c r="B37" s="83" t="s">
+        <v>619</v>
+      </c>
+      <c r="C37" s="83" t="s">
+        <v>589</v>
+      </c>
+      <c r="D37" s="84">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="81" t="s">
+        <v>309</v>
+      </c>
+      <c r="B38" s="81" t="s">
+        <v>620</v>
+      </c>
+      <c r="C38" s="81" t="s">
+        <v>600</v>
+      </c>
+      <c r="D38" s="82">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="83" t="s">
+        <v>290</v>
+      </c>
+      <c r="B39" s="83" t="s">
+        <v>621</v>
+      </c>
+      <c r="C39" s="83" t="s">
+        <v>600</v>
+      </c>
+      <c r="D39" s="84">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="81" t="s">
+        <v>159</v>
+      </c>
+      <c r="B40" s="81" t="s">
+        <v>622</v>
+      </c>
+      <c r="C40" s="81" t="s">
+        <v>596</v>
+      </c>
+      <c r="D40" s="82">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="83" t="s">
+        <v>452</v>
+      </c>
+      <c r="B41" s="83" t="s">
+        <v>623</v>
+      </c>
+      <c r="C41" s="83" t="s">
+        <v>593</v>
+      </c>
+      <c r="D41" s="84">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="81" t="s">
+        <v>430</v>
+      </c>
+      <c r="B42" s="81" t="s">
+        <v>624</v>
+      </c>
+      <c r="C42" s="81" t="s">
+        <v>589</v>
+      </c>
+      <c r="D42" s="82">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="83" t="s">
+        <v>426</v>
+      </c>
+      <c r="B43" s="83" t="s">
+        <v>625</v>
+      </c>
+      <c r="C43" s="83" t="s">
+        <v>589</v>
+      </c>
+      <c r="D43" s="84">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="81" t="s">
+        <v>428</v>
+      </c>
+      <c r="B44" s="81" t="s">
+        <v>626</v>
+      </c>
+      <c r="C44" s="81" t="s">
+        <v>589</v>
+      </c>
+      <c r="D44" s="82">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" s="83" t="s">
+        <v>627</v>
+      </c>
+      <c r="C45" s="83" t="s">
+        <v>578</v>
+      </c>
+      <c r="D45" s="84">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="81" t="s">
+        <v>628</v>
+      </c>
+      <c r="B46" s="81" t="s">
+        <v>629</v>
+      </c>
+      <c r="C46" s="81" t="s">
+        <v>630</v>
+      </c>
+      <c r="D46" s="82">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="83" t="s">
+        <v>155</v>
+      </c>
+      <c r="B47" s="83" t="s">
+        <v>631</v>
+      </c>
+      <c r="C47" s="83" t="s">
+        <v>596</v>
+      </c>
+      <c r="D47" s="84">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="81" t="s">
+        <v>632</v>
+      </c>
+      <c r="B48" s="81" t="s">
+        <v>633</v>
+      </c>
+      <c r="C48" s="81" t="s">
+        <v>574</v>
+      </c>
+      <c r="D48" s="82">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="83" t="s">
+        <v>634</v>
+      </c>
+      <c r="B49" s="83" t="s">
+        <v>635</v>
+      </c>
+      <c r="C49" s="83" t="s">
+        <v>574</v>
+      </c>
+      <c r="D49" s="84">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="81" t="s">
+        <v>509</v>
+      </c>
+      <c r="B50" s="81" t="s">
+        <v>636</v>
+      </c>
+      <c r="C50" s="81" t="s">
+        <v>602</v>
+      </c>
+      <c r="D50" s="82">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="83" t="s">
+        <v>88</v>
+      </c>
+      <c r="B51" s="83" t="s">
+        <v>637</v>
+      </c>
+      <c r="C51" s="83" t="s">
+        <v>578</v>
+      </c>
+      <c r="D51" s="84">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="81" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" s="81" t="s">
+        <v>638</v>
+      </c>
+      <c r="C52" s="81" t="s">
+        <v>578</v>
+      </c>
+      <c r="D52" s="82">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="83" t="s">
+        <v>639</v>
+      </c>
+      <c r="B53" s="83" t="s">
+        <v>640</v>
+      </c>
+      <c r="C53" s="83" t="s">
+        <v>574</v>
+      </c>
+      <c r="D53" s="84">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="81" t="s">
+        <v>161</v>
+      </c>
+      <c r="B54" s="81" t="s">
+        <v>641</v>
+      </c>
+      <c r="C54" s="81" t="s">
+        <v>589</v>
+      </c>
+      <c r="D54" s="82">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="83" t="s">
+        <v>642</v>
+      </c>
+      <c r="B55" s="83" t="s">
+        <v>643</v>
+      </c>
+      <c r="C55" s="83" t="s">
+        <v>574</v>
+      </c>
+      <c r="D55" s="84">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="81" t="s">
+        <v>292</v>
+      </c>
+      <c r="B56" s="81" t="s">
+        <v>644</v>
+      </c>
+      <c r="C56" s="81" t="s">
+        <v>600</v>
+      </c>
+      <c r="D56" s="82">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="83" t="s">
+        <v>645</v>
+      </c>
+      <c r="B57" s="83" t="s">
+        <v>646</v>
+      </c>
+      <c r="C57" s="83" t="s">
+        <v>647</v>
+      </c>
+      <c r="D57" s="84">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="81" t="s">
+        <v>92</v>
+      </c>
+      <c r="B58" s="81" t="s">
+        <v>648</v>
+      </c>
+      <c r="C58" s="81" t="s">
+        <v>578</v>
+      </c>
+      <c r="D58" s="82">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="83" t="s">
+        <v>472</v>
+      </c>
+      <c r="B59" s="83" t="s">
+        <v>649</v>
+      </c>
+      <c r="C59" s="83" t="s">
+        <v>630</v>
+      </c>
+      <c r="D59" s="84">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="81" t="s">
+        <v>467</v>
+      </c>
+      <c r="B60" s="81" t="s">
+        <v>650</v>
+      </c>
+      <c r="C60" s="81" t="s">
+        <v>630</v>
+      </c>
+      <c r="D60" s="82">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="83" t="s">
+        <v>651</v>
+      </c>
+      <c r="B61" s="83" t="s">
+        <v>652</v>
+      </c>
+      <c r="C61" s="83" t="s">
+        <v>647</v>
+      </c>
+      <c r="D61" s="84">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="81" t="s">
+        <v>653</v>
+      </c>
+      <c r="B62" s="81" t="s">
+        <v>654</v>
+      </c>
+      <c r="C62" s="81" t="s">
+        <v>647</v>
+      </c>
+      <c r="D62" s="82">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="83" t="s">
+        <v>655</v>
+      </c>
+      <c r="B63" s="83" t="s">
+        <v>656</v>
+      </c>
+      <c r="C63" s="83" t="s">
+        <v>647</v>
+      </c>
+      <c r="D63" s="84">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="81" t="s">
+        <v>157</v>
+      </c>
+      <c r="B64" s="81" t="s">
+        <v>657</v>
+      </c>
+      <c r="C64" s="81" t="s">
+        <v>596</v>
+      </c>
+      <c r="D64" s="82">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="83" t="s">
+        <v>450</v>
+      </c>
+      <c r="B65" s="83" t="s">
+        <v>658</v>
+      </c>
+      <c r="C65" s="83" t="s">
+        <v>593</v>
+      </c>
+      <c r="D65" s="84">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="81" t="s">
+        <v>659</v>
+      </c>
+      <c r="B66" s="81" t="s">
+        <v>660</v>
+      </c>
+      <c r="C66" s="81" t="s">
+        <v>630</v>
+      </c>
+      <c r="D66" s="82">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="83" t="s">
+        <v>513</v>
+      </c>
+      <c r="B67" s="83" t="s">
+        <v>661</v>
+      </c>
+      <c r="C67" s="83" t="s">
+        <v>602</v>
+      </c>
+      <c r="D67" s="84">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="81" t="s">
+        <v>662</v>
+      </c>
+      <c r="B68" s="81" t="s">
+        <v>663</v>
+      </c>
+      <c r="C68" s="81" t="s">
+        <v>647</v>
+      </c>
+      <c r="D68" s="82">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="83" t="s">
+        <v>664</v>
+      </c>
+      <c r="B69" s="83" t="s">
+        <v>665</v>
+      </c>
+      <c r="C69" s="83" t="s">
+        <v>647</v>
+      </c>
+      <c r="D69" s="84">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="81" t="s">
+        <v>666</v>
+      </c>
+      <c r="B70" s="81" t="s">
+        <v>667</v>
+      </c>
+      <c r="C70" s="81" t="s">
+        <v>647</v>
+      </c>
+      <c r="D70" s="82">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="83" t="s">
+        <v>668</v>
+      </c>
+      <c r="B71" s="83" t="s">
+        <v>669</v>
+      </c>
+      <c r="C71" s="83" t="s">
+        <v>647</v>
+      </c>
+      <c r="D71" s="84">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="85" t="s">
         <v>267</v>
       </c>
-      <c r="B18" s="85" t="s">
-        <v>596</v>
-      </c>
-      <c r="C18" s="85" t="s">
+      <c r="B72" s="85" t="s">
+        <v>670</v>
+      </c>
+      <c r="C72" s="85" t="s">
         <v>267</v>
       </c>
-      <c r="D18" s="86">
-        <v>7873</v>
+      <c r="D72" s="86">
+        <v>56233</v>
       </c>
     </row>
   </sheetData>
@@ -24802,44 +25768,44 @@
         <v>66</v>
       </c>
       <c r="C1" s="87" t="s">
-        <v>597</v>
+        <v>671</v>
       </c>
       <c r="D1" s="87" t="s">
-        <v>598</v>
+        <v>672</v>
       </c>
       <c r="E1" s="87" t="s">
-        <v>599</v>
+        <v>673</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="88" t="s">
-        <v>434</v>
+        <v>459</v>
       </c>
       <c r="B2" s="88" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="C2" s="89">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D2" s="90">
-        <v>46</v>
+        <v>43.3</v>
       </c>
       <c r="E2" s="91">
-        <v>0.52</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="88" t="s">
-        <v>586</v>
+        <v>434</v>
       </c>
       <c r="B3" s="88" t="s">
-        <v>587</v>
+        <v>619</v>
       </c>
       <c r="C3" s="89">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D3" s="90">
-        <v>1.9</v>
+        <v>46</v>
       </c>
       <c r="E3" s="91">
         <v>0.52</v>
@@ -24847,36 +25813,36 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="88" t="s">
-        <v>338</v>
+        <v>655</v>
       </c>
       <c r="B4" s="88" t="s">
-        <v>601</v>
+        <v>656</v>
       </c>
       <c r="C4" s="89">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="90">
-        <v>6.8</v>
+        <v>1.9</v>
       </c>
       <c r="E4" s="91">
-        <v>0.59</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="88" t="s">
-        <v>459</v>
+        <v>338</v>
       </c>
       <c r="B5" s="88" t="s">
-        <v>602</v>
+        <v>674</v>
       </c>
       <c r="C5" s="89">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D5" s="90">
-        <v>43.3</v>
+        <v>6.8</v>
       </c>
       <c r="E5" s="91">
-        <v>0.67</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -24884,7 +25850,7 @@
         <v>391</v>
       </c>
       <c r="B6" s="92" t="s">
-        <v>603</v>
+        <v>675</v>
       </c>
       <c r="C6" s="93">
         <v>53</v>
@@ -24901,7 +25867,7 @@
         <v>393</v>
       </c>
       <c r="B7" s="92" t="s">
-        <v>604</v>
+        <v>676</v>
       </c>
       <c r="C7" s="93">
         <v>56</v>
@@ -24918,7 +25884,7 @@
         <v>388</v>
       </c>
       <c r="B8" s="92" t="s">
-        <v>605</v>
+        <v>677</v>
       </c>
       <c r="C8" s="93">
         <v>58</v>
@@ -24935,7 +25901,7 @@
         <v>416</v>
       </c>
       <c r="B9" s="92" t="s">
-        <v>606</v>
+        <v>618</v>
       </c>
       <c r="C9" s="93">
         <v>33</v>
@@ -24952,7 +25918,7 @@
         <v>372</v>
       </c>
       <c r="B10" s="92" t="s">
-        <v>607</v>
+        <v>678</v>
       </c>
       <c r="C10" s="93">
         <v>86</v>
@@ -24969,7 +25935,7 @@
         <v>491</v>
       </c>
       <c r="B11" s="92" t="s">
-        <v>608</v>
+        <v>679</v>
       </c>
       <c r="C11" s="93">
         <v>39</v>
@@ -24986,7 +25952,7 @@
         <v>374</v>
       </c>
       <c r="B12" s="92" t="s">
-        <v>609</v>
+        <v>680</v>
       </c>
       <c r="C12" s="93">
         <v>40</v>
@@ -25003,7 +25969,7 @@
         <v>426</v>
       </c>
       <c r="B13" s="92" t="s">
-        <v>610</v>
+        <v>625</v>
       </c>
       <c r="C13" s="93">
         <v>77</v>
@@ -25020,7 +25986,7 @@
         <v>370</v>
       </c>
       <c r="B14" s="92" t="s">
-        <v>611</v>
+        <v>681</v>
       </c>
       <c r="C14" s="93">
         <v>100</v>
@@ -25037,7 +26003,7 @@
         <v>364</v>
       </c>
       <c r="B15" s="92" t="s">
-        <v>612</v>
+        <v>682</v>
       </c>
       <c r="C15" s="93">
         <v>100</v>
@@ -25054,7 +26020,7 @@
         <v>495</v>
       </c>
       <c r="B16" s="92" t="s">
-        <v>613</v>
+        <v>683</v>
       </c>
       <c r="C16" s="93">
         <v>51</v>
@@ -25071,7 +26037,7 @@
         <v>384</v>
       </c>
       <c r="B17" s="92" t="s">
-        <v>614</v>
+        <v>684</v>
       </c>
       <c r="C17" s="93">
         <v>80</v>

</xml_diff>